<commit_message>
Validacao dados gold e silver
</commit_message>
<xml_diff>
--- a/TestDIR/Project_Pandas_2026_10_04_market/Raw/table_silver/SilverCadastro_ETL.xlsx
+++ b/TestDIR/Project_Pandas_2026_10_04_market/Raw/table_silver/SilverCadastro_ETL.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H23"/>
+  <dimension ref="A1:H25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1162,6 +1162,54 @@
         </is>
       </c>
     </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>1000001</v>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>N_INFO</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>N_INFO</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr"/>
+      <c r="E24" t="inlineStr"/>
+      <c r="F24" t="inlineStr"/>
+      <c r="G24" t="inlineStr"/>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>N_INFO</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
+        <v>999</v>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>N_INFO</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>N_INFO</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr"/>
+      <c r="E25" t="inlineStr"/>
+      <c r="F25" t="inlineStr"/>
+      <c r="G25" t="inlineStr"/>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>N_INFO</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>